<commit_message>
A Days work, fixing and making mistakes, new figures , a good start on tables
</commit_message>
<xml_diff>
--- a/Tables/OSRI_Table1.xlsx
+++ b/Tables/OSRI_Table1.xlsx
@@ -424,7 +424,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Seaweed</t>
+          <t>Clams</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -438,7 +438,7 @@
         </is>
       </c>
       <c r="F2">
-        <v>28</v>
+        <v>77</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
@@ -446,32 +446,32 @@
         </is>
       </c>
       <c r="H2">
-        <v>5.161</v>
+        <v>89.3</v>
       </c>
       <c r="I2">
         <v>0.5600000000000001</v>
       </c>
       <c r="J2">
-        <v>0.9578928571428572</v>
+        <v>11.88435064935065</v>
       </c>
       <c r="K2">
-        <v>0.5600000000000001</v>
+        <v>4.11</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Arnold</t>
+          <t>Diver</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Public Health Evaluation following Selendang AYU, Arnold</t>
+          <t>NOAA Western Mariner Assessment</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Snails</t>
+          <t>Clams</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -485,24 +485,24 @@
         </is>
       </c>
       <c r="F3">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2005 - 2005</t>
+          <t>2022 - 2023</t>
         </is>
       </c>
       <c r="H3">
-        <v>1882</v>
+        <v>34.21</v>
       </c>
       <c r="I3">
-        <v>7.1</v>
+        <v>2.694</v>
       </c>
       <c r="J3">
-        <v>222.2235294117647</v>
+        <v>7.713480000000001</v>
       </c>
       <c r="K3">
-        <v>16</v>
+        <v>4.82</v>
       </c>
     </row>
     <row r="4">
@@ -513,12 +513,12 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>NOAA Metlakatla Annette Islands Biota Study</t>
+          <t>NOAA AKMAP Special Study</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Snails</t>
+          <t>Clams</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -532,40 +532,40 @@
         </is>
       </c>
       <c r="F4">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2002 - 2002</t>
+          <t>2007 - 2008</t>
         </is>
       </c>
       <c r="H4">
-        <v>10.35</v>
+        <v>3.621</v>
       </c>
       <c r="I4">
-        <v>0.5600000000000001</v>
+        <v>1.872</v>
       </c>
       <c r="J4">
-        <v>1.633</v>
+        <v>2.969666666666666</v>
       </c>
       <c r="K4">
-        <v>0.5600000000000001</v>
+        <v>3.1005</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Harvey</t>
+          <t>Diver</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Chukchi Sea Whelks, Harvey</t>
+          <t>NOAA Mussel Watch</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Snails</t>
+          <t>Clams</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -579,40 +579,40 @@
         </is>
       </c>
       <c r="F5">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2009 - 2009</t>
+          <t>2007 - 2008</t>
         </is>
       </c>
       <c r="H5">
-        <v>10.7</v>
+        <v>10.36892</v>
       </c>
       <c r="I5">
-        <v>4.47</v>
+        <v>1.17</v>
       </c>
       <c r="J5">
-        <v>6.779999999999999</v>
+        <v>5.76946</v>
       </c>
       <c r="K5">
-        <v>5.17</v>
+        <v>5.76946</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Ma</t>
+          <t>Diver</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Bering and Chukchi Sea Sampling, Ma</t>
+          <t>NOAA North Pacific Research Board Study</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Snails</t>
+          <t>Clams</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -626,45 +626,45 @@
         </is>
       </c>
       <c r="F6">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2014 - 2014</t>
+          <t>2010 - 2010</t>
         </is>
       </c>
       <c r="H6">
-        <v>48.09</v>
+        <v>25.884</v>
       </c>
       <c r="I6">
-        <v>40.65</v>
+        <v>16.434</v>
       </c>
       <c r="J6">
-        <v>44.37</v>
+        <v>20.782</v>
       </c>
       <c r="K6">
-        <v>44.37</v>
+        <v>21.165</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Selendang</t>
+          <t>NCCOS</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Seledang AYU Post Spill Monitoring</t>
+          <t>NOAA Resurrection Bay Project</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Snails</t>
+          <t>Clams</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Post-oil spill assessment</t>
+          <t>Background biomonitoring</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -673,45 +673,45 @@
         </is>
       </c>
       <c r="F7">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2005 - 2005</t>
+          <t>2009 - 2010</t>
         </is>
       </c>
       <c r="H7">
-        <v>1481.74</v>
+        <v>225.8</v>
       </c>
       <c r="I7">
-        <v>1481.74</v>
+        <v>88.20000000000002</v>
       </c>
       <c r="J7">
-        <v>1481.74</v>
+        <v>149.6888888888889</v>
       </c>
       <c r="K7">
-        <v>1481.74</v>
+        <v>145.8</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Arnold</t>
+          <t>Shigenaka</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Public Health Evaluation following Selendang AYU, Arnold</t>
+          <t>Exxon Valdez Intertidal Study, Shigenaka</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Urchins/ Starfish</t>
+          <t>Clams</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Post-oil spill assessment</t>
+          <t>Background biomonitoring / Post-oil spill assessment</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -720,40 +720,40 @@
         </is>
       </c>
       <c r="F8">
-        <v>12</v>
+        <v>22</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>2005 - 2005</t>
+          <t>2007 - 2007</t>
         </is>
       </c>
       <c r="H8">
-        <v>120</v>
+        <v>373</v>
       </c>
       <c r="I8">
-        <v>6</v>
+        <v>6.2</v>
       </c>
       <c r="J8">
-        <v>39.15833333333333</v>
+        <v>86.2</v>
       </c>
       <c r="K8">
-        <v>13.5</v>
+        <v>23.5</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Ma</t>
+          <t>Diver</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Bering and Chukchi Sea Sampling, Ma</t>
+          <t>NOAA Metlakatla Annette Islands Biota Study</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Urchins/ Starfish</t>
+          <t>Crabs/ Shrimp</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -767,87 +767,87 @@
         </is>
       </c>
       <c r="F9">
-        <v>2</v>
+        <v>18</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>2014 - 2014</t>
+          <t>2002 - 2002</t>
         </is>
       </c>
       <c r="H9">
-        <v>118.38</v>
+        <v>5900</v>
       </c>
       <c r="I9">
-        <v>47.54</v>
+        <v>1.38</v>
       </c>
       <c r="J9">
-        <v>82.95999999999999</v>
+        <v>1266.380444444444</v>
       </c>
       <c r="K9">
-        <v>82.95999999999999</v>
+        <v>14.214</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Selendang</t>
+          <t>Diver</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Seledang AYU Post Spill Monitoring</t>
+          <t>NOAA Mussel Watch</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Urchins/ Starfish</t>
+          <t>Crabs/ Shrimp</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Post-oil spill assessment</t>
+          <t>Background biomonitoring</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Calculated</t>
+          <t>Provided</t>
         </is>
       </c>
       <c r="F10">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>2005 - 2005</t>
+          <t>2008 - 2008</t>
         </is>
       </c>
       <c r="H10">
-        <v>117.2</v>
+        <v>6.81992</v>
       </c>
       <c r="I10">
-        <v>15.71</v>
+        <v>6.81992</v>
       </c>
       <c r="J10">
-        <v>76.86000000000001</v>
+        <v>6.81992</v>
       </c>
       <c r="K10">
-        <v>87.26500000000001</v>
+        <v>6.81992</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Diver</t>
+          <t>Ma</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>NOAA Metlakatla Annette Islands Biota Study</t>
+          <t>Bering and Chukchi Sea Sampling, Ma</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Octopus</t>
+          <t>Crabs/ Shrimp</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -861,40 +861,40 @@
         </is>
       </c>
       <c r="F11">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>2002 - 2002</t>
+          <t>2014 - 2014</t>
         </is>
       </c>
       <c r="H11">
-        <v>35.25</v>
+        <v>72.88</v>
       </c>
       <c r="I11">
-        <v>0.5600000000000001</v>
+        <v>67.91</v>
       </c>
       <c r="J11">
-        <v>11.93428571428571</v>
+        <v>70.395</v>
       </c>
       <c r="K11">
-        <v>4.67</v>
+        <v>70.395</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Diver</t>
+          <t>Wetzel</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>NOAA Metlakatla Annette Islands Biota Study</t>
+          <t>Mote Marine Laboratory</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Clams</t>
+          <t>Crabs/ Shrimp</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -908,40 +908,40 @@
         </is>
       </c>
       <c r="F12">
-        <v>77</v>
+        <v>10</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>2002 - 2002</t>
+          <t>2012 - 2012</t>
         </is>
       </c>
       <c r="H12">
-        <v>89.3</v>
+        <v>0</v>
       </c>
       <c r="I12">
-        <v>0.5600000000000001</v>
+        <v>0</v>
       </c>
       <c r="J12">
-        <v>11.88435064935065</v>
+        <v>0</v>
       </c>
       <c r="K12">
-        <v>4.11</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Diver</t>
+          <t>Arnold</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>NOAA Western Mariner Assessment</t>
+          <t>Public Health Evaluation following Selendang AYU, Arnold</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Clams</t>
+          <t>Fish</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -955,24 +955,24 @@
         </is>
       </c>
       <c r="F13">
-        <v>25</v>
+        <v>7</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>2022 - 2023</t>
+          <t>2005 - 2005</t>
         </is>
       </c>
       <c r="H13">
-        <v>34.21</v>
+        <v>17</v>
       </c>
       <c r="I13">
-        <v>2.694</v>
+        <v>4.8</v>
       </c>
       <c r="J13">
-        <v>7.713480000000001</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="K13">
-        <v>4.82</v>
+        <v>7.1</v>
       </c>
     </row>
     <row r="14">
@@ -983,12 +983,12 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>NOAA AKMAP Special Study</t>
+          <t>NOAA Metlakatla Annette Islands Biota Study</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Clams</t>
+          <t>Fish</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -1002,24 +1002,24 @@
         </is>
       </c>
       <c r="F14">
-        <v>6</v>
+        <v>17</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>2007 - 2008</t>
+          <t>2002 - 2002</t>
         </is>
       </c>
       <c r="H14">
-        <v>3.621</v>
+        <v>30.29</v>
       </c>
       <c r="I14">
-        <v>1.872</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="J14">
-        <v>2.969666666666666</v>
+        <v>9.001764705882353</v>
       </c>
       <c r="K14">
-        <v>3.1005</v>
+        <v>5.41</v>
       </c>
     </row>
     <row r="15">
@@ -1030,17 +1030,17 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>NOAA Mussel Watch</t>
+          <t>NOAA Western Mariner Assessment</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Clams</t>
+          <t>Fish</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Background biomonitoring</t>
+          <t>Post-oil spill assessment</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -1049,40 +1049,40 @@
         </is>
       </c>
       <c r="F15">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>2007 - 2008</t>
+          <t>2022 - 2022</t>
         </is>
       </c>
       <c r="H15">
-        <v>10.36892</v>
+        <v>10.374</v>
       </c>
       <c r="I15">
-        <v>1.17</v>
+        <v>2.72</v>
       </c>
       <c r="J15">
-        <v>5.76946</v>
+        <v>4.9885</v>
       </c>
       <c r="K15">
-        <v>5.76946</v>
+        <v>3.839</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Diver</t>
+          <t>ERM</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>NOAA North Pacific Research Board Study</t>
+          <t>North Slope Subsistence Study</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Clams</t>
+          <t>Fish</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -1092,44 +1092,44 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Provided</t>
+          <t>Calculated</t>
         </is>
       </c>
       <c r="F16">
-        <v>5</v>
+        <v>110</v>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>2010 - 2010</t>
+          <t>2014 - 2015</t>
         </is>
       </c>
       <c r="H16">
-        <v>25.884</v>
+        <v>96.59999999999999</v>
       </c>
       <c r="I16">
-        <v>16.434</v>
+        <v>0</v>
       </c>
       <c r="J16">
-        <v>20.782</v>
+        <v>8.063136363636366</v>
       </c>
       <c r="K16">
-        <v>21.165</v>
+        <v>3.525</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>NCCOS</t>
+          <t>Ma</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>NOAA Resurrection Bay Project</t>
+          <t>Bering and Chukchi Sea Sampling, Ma</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Clams</t>
+          <t>Fish</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -1139,143 +1139,143 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Calculated</t>
+          <t>Provided</t>
         </is>
       </c>
       <c r="F17">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>2009 - 2010</t>
+          <t>2014 - 2014</t>
         </is>
       </c>
       <c r="H17">
-        <v>225.8</v>
+        <v>128.07</v>
       </c>
       <c r="I17">
-        <v>88.20000000000002</v>
+        <v>36.1</v>
       </c>
       <c r="J17">
-        <v>149.6888888888889</v>
+        <v>78.91</v>
       </c>
       <c r="K17">
-        <v>145.8</v>
+        <v>75.735</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Shigenaka</t>
+          <t>NCCOS</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Exxon Valdez Intertidal Study, Shigenaka</t>
+          <t>NOAA Bristol Bay Study</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Clams</t>
+          <t>Fish</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Background biomonitoring / Post-oil spill assessment</t>
+          <t>Background biomonitoring</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Provided</t>
+          <t>Calculated</t>
         </is>
       </c>
       <c r="F18">
-        <v>22</v>
+        <v>10</v>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>2007 - 2007</t>
+          <t>2013 - 2014</t>
         </is>
       </c>
       <c r="H18">
-        <v>373</v>
+        <v>160.411</v>
       </c>
       <c r="I18">
-        <v>6.2</v>
+        <v>27.029</v>
       </c>
       <c r="J18">
-        <v>86.2</v>
+        <v>62.4798</v>
       </c>
       <c r="K18">
-        <v>23.5</v>
+        <v>51.53450000000001</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Arnold</t>
+          <t>NCCOS</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Public Health Evaluation following Selendang AYU, Arnold</t>
+          <t>NOAA Alaska Arctic Study</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Mussels</t>
+          <t>Fish</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Post-oil spill assessment</t>
+          <t>Background biomonitoring</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Provided</t>
+          <t>Calculated</t>
         </is>
       </c>
       <c r="F19">
-        <v>30</v>
+        <v>4</v>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>2005 - 2005</t>
+          <t>2015 - 2015</t>
         </is>
       </c>
       <c r="H19">
-        <v>7759</v>
+        <v>113.561</v>
       </c>
       <c r="I19">
-        <v>7.1</v>
+        <v>52.647</v>
       </c>
       <c r="J19">
-        <v>678.5833333333334</v>
+        <v>89.816</v>
       </c>
       <c r="K19">
-        <v>74.5</v>
+        <v>96.52800000000002</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Diver</t>
+          <t>Wetzel</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>NOAA Western Mariner Assessment</t>
+          <t>Mote Marine Laboratory</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Mussels</t>
+          <t>Fish</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Post-oil spill assessment</t>
+          <t>Background biomonitoring</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -1284,35 +1284,35 @@
         </is>
       </c>
       <c r="F20">
-        <v>46</v>
+        <v>552</v>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>2022 - 2024</t>
+          <t>2005 - 2024</t>
         </is>
       </c>
       <c r="H20">
-        <v>222.08</v>
+        <v>118480</v>
       </c>
       <c r="I20">
-        <v>2.87</v>
+        <v>0</v>
       </c>
       <c r="J20">
-        <v>17.55430434782609</v>
+        <v>1032.568255293754</v>
       </c>
       <c r="K20">
-        <v>5.6</v>
+        <v>0</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Diver</t>
+          <t>Arnold</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>NOAA AKMAP Special Study</t>
+          <t>Public Health Evaluation following Selendang AYU, Arnold</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -1322,7 +1322,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Background biomonitoring</t>
+          <t>Post-oil spill assessment</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -1331,24 +1331,24 @@
         </is>
       </c>
       <c r="F21">
-        <v>12</v>
+        <v>30</v>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>2007 - 2008</t>
+          <t>2005 - 2005</t>
         </is>
       </c>
       <c r="H21">
-        <v>220.014</v>
+        <v>7759</v>
       </c>
       <c r="I21">
-        <v>7.308</v>
+        <v>7.1</v>
       </c>
       <c r="J21">
-        <v>34.45491666666667</v>
+        <v>678.5833333333334</v>
       </c>
       <c r="K21">
-        <v>11.725</v>
+        <v>74.5</v>
       </c>
     </row>
     <row r="22">
@@ -1359,7 +1359,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>NOAA Mussel Watch</t>
+          <t>NOAA Western Mariner Assessment</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1369,7 +1369,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Background biomonitoring</t>
+          <t>Post-oil spill assessment</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -1378,24 +1378,24 @@
         </is>
       </c>
       <c r="F22">
-        <v>34</v>
+        <v>46</v>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>2001 - 2009</t>
+          <t>2022 - 2024</t>
         </is>
       </c>
       <c r="H22">
-        <v>110.17114284</v>
+        <v>222.08</v>
       </c>
       <c r="I22">
-        <v>5.19093</v>
+        <v>2.87</v>
       </c>
       <c r="J22">
-        <v>17.51721504176471</v>
+        <v>17.55430434782609</v>
       </c>
       <c r="K22">
-        <v>13.028975</v>
+        <v>5.6</v>
       </c>
     </row>
     <row r="23">
@@ -1406,7 +1406,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>NOAA Pribilofs Special Study</t>
+          <t>NOAA AKMAP Special Study</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1425,35 +1425,35 @@
         </is>
       </c>
       <c r="F23">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>2000 - 2000</t>
+          <t>2007 - 2008</t>
         </is>
       </c>
       <c r="H23">
-        <v>1614.813</v>
+        <v>220.014</v>
       </c>
       <c r="I23">
-        <v>18.08</v>
+        <v>7.308</v>
       </c>
       <c r="J23">
-        <v>769.5002500000001</v>
+        <v>34.45491666666667</v>
       </c>
       <c r="K23">
-        <v>722.554</v>
+        <v>11.725</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Ma</t>
+          <t>Diver</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Bering and Chukchi Sea Sampling, Ma</t>
+          <t>NOAA Mussel Watch</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1472,35 +1472,35 @@
         </is>
       </c>
       <c r="F24">
-        <v>2</v>
+        <v>34</v>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>2014 - 2014</t>
+          <t>2001 - 2009</t>
         </is>
       </c>
       <c r="H24">
-        <v>86.68000000000001</v>
+        <v>110.17114284</v>
       </c>
       <c r="I24">
-        <v>34.18</v>
+        <v>5.19093</v>
       </c>
       <c r="J24">
-        <v>60.43000000000001</v>
+        <v>17.51721504176471</v>
       </c>
       <c r="K24">
-        <v>60.43000000000001</v>
+        <v>13.028975</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>NCCOS</t>
+          <t>Diver</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Alaska NPS Mussel Watch</t>
+          <t>NOAA Pribilofs Special Study</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1515,39 +1515,39 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Calculated</t>
+          <t>Provided</t>
         </is>
       </c>
       <c r="F25">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>2013 - 2013</t>
+          <t>2000 - 2000</t>
         </is>
       </c>
       <c r="H25">
-        <v>302.5399999999999</v>
+        <v>1614.813</v>
       </c>
       <c r="I25">
-        <v>25.617</v>
+        <v>18.08</v>
       </c>
       <c r="J25">
-        <v>84.16966666666666</v>
+        <v>769.5002500000001</v>
       </c>
       <c r="K25">
-        <v>44.039</v>
+        <v>722.554</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>NCCOS</t>
+          <t>Ma</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Long Term Monitoring Gulf Watch</t>
+          <t>Bering and Chukchi Sea Sampling, Ma</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1562,28 +1562,28 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Calculated</t>
+          <t>Provided</t>
         </is>
       </c>
       <c r="F26">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>2013 - 2013</t>
+          <t>2014 - 2014</t>
         </is>
       </c>
       <c r="H26">
-        <v>58.748</v>
+        <v>86.68000000000001</v>
       </c>
       <c r="I26">
-        <v>52.01199999999999</v>
+        <v>34.18</v>
       </c>
       <c r="J26">
-        <v>55.01966666666666</v>
+        <v>60.43000000000001</v>
       </c>
       <c r="K26">
-        <v>54.29899999999999</v>
+        <v>60.43000000000001</v>
       </c>
     </row>
     <row r="27">
@@ -1594,7 +1594,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>NOAA Southwest Alaska Nearshore Monitoring</t>
+          <t>Alaska NPS Mussel Watch</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1613,24 +1613,24 @@
         </is>
       </c>
       <c r="F27">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>2007 - 2007</t>
+          <t>2013 - 2013</t>
         </is>
       </c>
       <c r="H27">
-        <v>98.70000000000003</v>
+        <v>302.5399999999999</v>
       </c>
       <c r="I27">
-        <v>65.90000000000001</v>
+        <v>25.617</v>
       </c>
       <c r="J27">
-        <v>81.04545454545455</v>
+        <v>84.16966666666666</v>
       </c>
       <c r="K27">
-        <v>77.2</v>
+        <v>44.039</v>
       </c>
     </row>
     <row r="28">
@@ -1641,7 +1641,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>NOAA Resurrection Bay Project</t>
+          <t>Long Term Monitoring Gulf Watch</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -1660,24 +1660,24 @@
         </is>
       </c>
       <c r="F28">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>2009 - 2010</t>
+          <t>2013 - 2013</t>
         </is>
       </c>
       <c r="H28">
-        <v>595.1000000000001</v>
+        <v>58.748</v>
       </c>
       <c r="I28">
-        <v>219.5</v>
+        <v>52.01199999999999</v>
       </c>
       <c r="J28">
-        <v>354.06</v>
+        <v>55.01966666666666</v>
       </c>
       <c r="K28">
-        <v>281.9</v>
+        <v>54.29899999999999</v>
       </c>
     </row>
     <row r="29">
@@ -1688,7 +1688,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>NOAA Kachemak Bay Bioeffects</t>
+          <t>NOAA Southwest Alaska Nearshore Monitoring</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -1707,35 +1707,35 @@
         </is>
       </c>
       <c r="F29">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>2009 - 2009</t>
+          <t>2007 - 2007</t>
         </is>
       </c>
       <c r="H29">
-        <v>455.6619999999999</v>
+        <v>98.70000000000003</v>
       </c>
       <c r="I29">
-        <v>157.505</v>
+        <v>65.90000000000001</v>
       </c>
       <c r="J29">
-        <v>306.5835</v>
+        <v>81.04545454545455</v>
       </c>
       <c r="K29">
-        <v>306.5835</v>
+        <v>77.2</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Nationwide</t>
+          <t>NCCOS</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>NOAA Mussel Watch</t>
+          <t>NOAA Resurrection Bay Project</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -1750,39 +1750,39 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Provided</t>
+          <t>Calculated</t>
         </is>
       </c>
       <c r="F30">
-        <v>24</v>
+        <v>5</v>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>2012 - 2012</t>
+          <t>2009 - 2010</t>
         </is>
       </c>
       <c r="H30">
-        <v>295.5</v>
+        <v>595.1000000000001</v>
       </c>
       <c r="I30">
-        <v>8.808</v>
+        <v>219.5</v>
       </c>
       <c r="J30">
-        <v>59.14858333333333</v>
+        <v>354.06</v>
       </c>
       <c r="K30">
-        <v>19.59</v>
+        <v>281.9</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>PWSRCAC</t>
+          <t>NCCOS</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Prince William Sound Regional Citizens' Advisory Council Monitoring</t>
+          <t>NOAA Kachemak Bay Bioeffects</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -1792,7 +1792,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Background biomonitoring / Post-oil spill assessment</t>
+          <t>Background biomonitoring</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -1801,35 +1801,35 @@
         </is>
       </c>
       <c r="F31">
-        <v>925</v>
+        <v>2</v>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>2000 - 2024</t>
+          <t>2009 - 2009</t>
         </is>
       </c>
       <c r="H31">
-        <v>97962.52972799999</v>
+        <v>455.6619999999999</v>
       </c>
       <c r="I31">
-        <v>1.4</v>
+        <v>157.505</v>
       </c>
       <c r="J31">
-        <v>873.2899081741966</v>
+        <v>306.5835</v>
       </c>
       <c r="K31">
-        <v>45.24285959999999</v>
+        <v>306.5835</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>PWSRCAC</t>
+          <t>Nationwide</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Prince William Sound Regional Citizens' Advisory Council Monitoring</t>
+          <t>NOAA Mussel Watch</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -1839,44 +1839,44 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Post-oil spill assessment</t>
+          <t>Background biomonitoring</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Calculated</t>
+          <t>Provided</t>
         </is>
       </c>
       <c r="F32">
-        <v>3</v>
+        <v>24</v>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>2020 - 2020</t>
+          <t>2012 - 2012</t>
         </is>
       </c>
       <c r="H32">
-        <v>244574.47847</v>
+        <v>295.5</v>
       </c>
       <c r="I32">
-        <v>158498.563017</v>
+        <v>8.808</v>
       </c>
       <c r="J32">
-        <v>189175.25249</v>
+        <v>59.14858333333333</v>
       </c>
       <c r="K32">
-        <v>164452.715983</v>
+        <v>19.59</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Selendang</t>
+          <t>PWSRCAC</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Seledang AYU Post Spill Monitoring</t>
+          <t>Prince William Sound Regional Citizens' Advisory Council Monitoring</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -1886,7 +1886,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Post-oil spill assessment</t>
+          <t>Background biomonitoring / Post-oil spill assessment</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -1895,50 +1895,50 @@
         </is>
       </c>
       <c r="F33">
-        <v>3</v>
+        <v>910</v>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>2005 - 2005</t>
+          <t>2000 - 2024</t>
         </is>
       </c>
       <c r="H33">
-        <v>10412.9</v>
+        <v>30038.6189051</v>
       </c>
       <c r="I33">
-        <v>233.42</v>
+        <v>1.4</v>
       </c>
       <c r="J33">
-        <v>5917.206666666667</v>
+        <v>205.8107942726725</v>
       </c>
       <c r="K33">
-        <v>7105.3</v>
+        <v>44.18354049999999</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Diver</t>
+          <t>PWSRCAC</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>NOAA Metlakatla Annette Islands Biota Study</t>
+          <t>Prince William Sound Regional Citizens' Advisory Council Monitoring</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Crabs/ Shrimp</t>
+          <t>Mussels</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Background biomonitoring</t>
+          <t>Post-oil spill assessment</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Provided</t>
+          <t>Calculated</t>
         </is>
       </c>
       <c r="F34">
@@ -1946,83 +1946,83 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>2002 - 2002</t>
+          <t>2020 - 2020</t>
         </is>
       </c>
       <c r="H34">
-        <v>5900</v>
+        <v>244574.47847</v>
       </c>
       <c r="I34">
-        <v>1.38</v>
+        <v>2136.01875</v>
       </c>
       <c r="J34">
-        <v>1266.380444444444</v>
+        <v>66001.72776349999</v>
       </c>
       <c r="K34">
-        <v>14.214</v>
+        <v>37082.8439115</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Diver</t>
+          <t>Selendang</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>NOAA Mussel Watch</t>
+          <t>Seledang AYU Post Spill Monitoring</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Crabs/ Shrimp</t>
+          <t>Mussels</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Background biomonitoring</t>
+          <t>Post-oil spill assessment</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Provided</t>
+          <t>Calculated</t>
         </is>
       </c>
       <c r="F35">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>2008 - 2008</t>
+          <t>2005 - 2005</t>
         </is>
       </c>
       <c r="H35">
-        <v>6.81992</v>
+        <v>10412.9</v>
       </c>
       <c r="I35">
-        <v>6.81992</v>
+        <v>233.42</v>
       </c>
       <c r="J35">
-        <v>6.81992</v>
+        <v>5917.206666666667</v>
       </c>
       <c r="K35">
-        <v>6.81992</v>
+        <v>7105.3</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Ma</t>
+          <t>Diver</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Bering and Chukchi Sea Sampling, Ma</t>
+          <t>NOAA Metlakatla Annette Islands Biota Study</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Crabs/ Shrimp</t>
+          <t>Octopus</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -2036,45 +2036,45 @@
         </is>
       </c>
       <c r="F36">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>2014 - 2014</t>
+          <t>2002 - 2002</t>
         </is>
       </c>
       <c r="H36">
-        <v>72.88</v>
+        <v>35.25</v>
       </c>
       <c r="I36">
-        <v>67.91</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="J36">
-        <v>70.395</v>
+        <v>11.93428571428571</v>
       </c>
       <c r="K36">
-        <v>70.395</v>
+        <v>4.67</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Wetzel</t>
+          <t>Arnold</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Mote Marine Laboratory</t>
+          <t>Public Health Evaluation following Selendang AYU, Arnold</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Crabs/ Shrimp</t>
+          <t>Seals/ Whales</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Background biomonitoring</t>
+          <t>Post-oil spill assessment</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -2083,45 +2083,45 @@
         </is>
       </c>
       <c r="F37">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>2012 - 2012</t>
+          <t>2005 - 2005</t>
         </is>
       </c>
       <c r="H37">
-        <v>0</v>
+        <v>18</v>
       </c>
       <c r="I37">
-        <v>0</v>
+        <v>18</v>
       </c>
       <c r="J37">
-        <v>0</v>
+        <v>18</v>
       </c>
       <c r="K37">
-        <v>0</v>
+        <v>18</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Arnold</t>
+          <t>Stimmelmayr</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Public Health Evaluation following Selendang AYU, Arnold</t>
+          <t>Oil Fouling of Seals, Stimmelmayr</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Fish</t>
+          <t>Seals/ Whales</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Post-oil spill assessment</t>
+          <t>Unknown oiling observed</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
@@ -2130,40 +2130,40 @@
         </is>
       </c>
       <c r="F38">
-        <v>7</v>
+        <v>30</v>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>2005 - 2005</t>
+          <t>2012 - 2014</t>
         </is>
       </c>
       <c r="H38">
-        <v>17</v>
+        <v>280</v>
       </c>
       <c r="I38">
-        <v>4.8</v>
+        <v>0</v>
       </c>
       <c r="J38">
-        <v>8.699999999999999</v>
+        <v>20.86333333333333</v>
       </c>
       <c r="K38">
-        <v>7.1</v>
+        <v>6.55</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Diver</t>
+          <t>Wetzel</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>NOAA Metlakatla Annette Islands Biota Study</t>
+          <t>Mote Marine Laboratory</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Fish</t>
+          <t>Seals/ Whales</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -2177,24 +2177,24 @@
         </is>
       </c>
       <c r="F39">
-        <v>17</v>
+        <v>276</v>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>2002 - 2002</t>
+          <t>2000 - 2016</t>
         </is>
       </c>
       <c r="H39">
-        <v>30.29</v>
+        <v>24329.77301543095</v>
       </c>
       <c r="I39">
-        <v>0.5600000000000001</v>
+        <v>0</v>
       </c>
       <c r="J39">
-        <v>9.001764705882353</v>
+        <v>1067.078335475072</v>
       </c>
       <c r="K39">
-        <v>5.41</v>
+        <v>0</v>
       </c>
     </row>
     <row r="40">
@@ -2205,17 +2205,17 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>NOAA Western Mariner Assessment</t>
+          <t>NOAA Metlakatla Annette Islands Biota Study</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Fish</t>
+          <t>Seaweed</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Post-oil spill assessment</t>
+          <t>Background biomonitoring</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
@@ -2224,87 +2224,87 @@
         </is>
       </c>
       <c r="F40">
-        <v>6</v>
+        <v>28</v>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>2022 - 2022</t>
+          <t>2002 - 2002</t>
         </is>
       </c>
       <c r="H40">
-        <v>10.374</v>
+        <v>5.161</v>
       </c>
       <c r="I40">
-        <v>2.72</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="J40">
-        <v>4.9885</v>
+        <v>0.9578928571428572</v>
       </c>
       <c r="K40">
-        <v>3.839</v>
+        <v>0.5600000000000001</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>ERM</t>
+          <t>Arnold</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>North Slope Subsistence Study</t>
+          <t>Public Health Evaluation following Selendang AYU, Arnold</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Fish</t>
+          <t>Snails</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Background biomonitoring</t>
+          <t>Post-oil spill assessment</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Calculated</t>
+          <t>Provided</t>
         </is>
       </c>
       <c r="F41">
-        <v>110</v>
+        <v>17</v>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>2014 - 2015</t>
+          <t>2005 - 2005</t>
         </is>
       </c>
       <c r="H41">
-        <v>0</v>
+        <v>1882</v>
       </c>
       <c r="I41">
-        <v>0</v>
+        <v>7.1</v>
       </c>
       <c r="J41">
-        <v>0</v>
+        <v>222.2235294117647</v>
       </c>
       <c r="K41">
-        <v>0</v>
+        <v>16</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Ma</t>
+          <t>Diver</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Bering and Chukchi Sea Sampling, Ma</t>
+          <t>NOAA Metlakatla Annette Islands Biota Study</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Fish</t>
+          <t>Snails</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -2318,40 +2318,40 @@
         </is>
       </c>
       <c r="F42">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>2014 - 2014</t>
+          <t>2002 - 2002</t>
         </is>
       </c>
       <c r="H42">
-        <v>128.07</v>
+        <v>10.35</v>
       </c>
       <c r="I42">
-        <v>36.1</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="J42">
-        <v>78.91</v>
+        <v>1.633</v>
       </c>
       <c r="K42">
-        <v>75.735</v>
+        <v>0.5600000000000001</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>NCCOS</t>
+          <t>Harvey</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>NOAA Bristol Bay Study</t>
+          <t>Chukchi Sea Whelks, Harvey</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Fish</t>
+          <t>Snails</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -2361,44 +2361,44 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Calculated</t>
+          <t>Provided</t>
         </is>
       </c>
       <c r="F43">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>2013 - 2014</t>
+          <t>2009 - 2009</t>
         </is>
       </c>
       <c r="H43">
-        <v>160.411</v>
+        <v>10.7</v>
       </c>
       <c r="I43">
-        <v>27.029</v>
+        <v>4.47</v>
       </c>
       <c r="J43">
-        <v>62.4798</v>
+        <v>6.779999999999999</v>
       </c>
       <c r="K43">
-        <v>51.53450000000001</v>
+        <v>5.17</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>NCCOS</t>
+          <t>Ma</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>NOAA Alaska Arctic Study</t>
+          <t>Bering and Chukchi Sea Sampling, Ma</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Fish</t>
+          <t>Snails</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -2408,75 +2408,75 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Calculated</t>
+          <t>Provided</t>
         </is>
       </c>
       <c r="F44">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>2015 - 2015</t>
+          <t>2014 - 2014</t>
         </is>
       </c>
       <c r="H44">
-        <v>113.561</v>
+        <v>48.09</v>
       </c>
       <c r="I44">
-        <v>52.647</v>
+        <v>40.65</v>
       </c>
       <c r="J44">
-        <v>89.816</v>
+        <v>44.37</v>
       </c>
       <c r="K44">
-        <v>96.52800000000002</v>
+        <v>44.37</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Wetzel</t>
+          <t>Selendang</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Mote Marine Laboratory</t>
+          <t>Seledang AYU Post Spill Monitoring</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Fish</t>
+          <t>Snails</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Background biomonitoring</t>
+          <t>Post-oil spill assessment</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Provided</t>
+          <t>Calculated</t>
         </is>
       </c>
       <c r="F45">
-        <v>552</v>
+        <v>1</v>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>2005 - 2024</t>
+          <t>2005 - 2005</t>
         </is>
       </c>
       <c r="H45">
-        <v>118480</v>
+        <v>1481.74</v>
       </c>
       <c r="I45">
-        <v>0</v>
+        <v>1481.74</v>
       </c>
       <c r="J45">
-        <v>1032.568255293754</v>
+        <v>1481.74</v>
       </c>
       <c r="K45">
-        <v>0</v>
+        <v>1481.74</v>
       </c>
     </row>
     <row r="46">
@@ -2492,7 +2492,7 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Seals/ Whales</t>
+          <t>Urchins/ Starfish</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -2506,7 +2506,7 @@
         </is>
       </c>
       <c r="F46">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="G46" t="inlineStr">
         <is>
@@ -2514,37 +2514,37 @@
         </is>
       </c>
       <c r="H46">
-        <v>18</v>
+        <v>120</v>
       </c>
       <c r="I46">
-        <v>18</v>
+        <v>6</v>
       </c>
       <c r="J46">
-        <v>18</v>
+        <v>39.15833333333333</v>
       </c>
       <c r="K46">
-        <v>18</v>
+        <v>13.5</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Stimmelmayr</t>
+          <t>Ma</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Oil Fouling of Seals, Stimmelmayr</t>
+          <t>Bering and Chukchi Sea Sampling, Ma</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Seals/ Whales</t>
+          <t>Urchins/ Starfish</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Unknown oiling observed</t>
+          <t>Background biomonitoring</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
@@ -2553,71 +2553,71 @@
         </is>
       </c>
       <c r="F47">
-        <v>30</v>
+        <v>2</v>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>2012 - 2014</t>
+          <t>2014 - 2014</t>
         </is>
       </c>
       <c r="H47">
-        <v>280</v>
+        <v>118.38</v>
       </c>
       <c r="I47">
-        <v>0</v>
+        <v>47.54</v>
       </c>
       <c r="J47">
-        <v>20.86333333333333</v>
+        <v>82.95999999999999</v>
       </c>
       <c r="K47">
-        <v>6.55</v>
+        <v>82.95999999999999</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Wetzel</t>
+          <t>Selendang</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Mote Marine Laboratory</t>
+          <t>Seledang AYU Post Spill Monitoring</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Seals/ Whales</t>
+          <t>Urchins/ Starfish</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Background biomonitoring</t>
+          <t>Post-oil spill assessment</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Provided</t>
+          <t>Calculated</t>
         </is>
       </c>
       <c r="F48">
-        <v>276</v>
+        <v>4</v>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>2000 - 2016</t>
+          <t>2005 - 2005</t>
         </is>
       </c>
       <c r="H48">
-        <v>24329.77301543095</v>
+        <v>117.2</v>
       </c>
       <c r="I48">
-        <v>0</v>
+        <v>15.71</v>
       </c>
       <c r="J48">
-        <v>1067.078335475072</v>
+        <v>76.86000000000001</v>
       </c>
       <c r="K48">
-        <v>0</v>
+        <v>87.26500000000001</v>
       </c>
     </row>
   </sheetData>

</xml_diff>